<commit_message>
collecting data for new experiment
</commit_message>
<xml_diff>
--- a/Experiment 1 - Testing Fixation Time/Time_for_Bac_Fix_Pos50_Mut49_Start.xlsx
+++ b/Experiment 1 - Testing Fixation Time/Time_for_Bac_Fix_Pos50_Mut49_Start.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Moar Documents\GitHub\Bac_Evol_SSA\Experiment 1 - Testing Fixation Time\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F3D4E6E-8035-45BA-9B46-0C30C87392D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C75E8CBB-0FE3-4CD9-BDF5-68519C96060C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{C5D5DF43-D68A-448F-BEE9-BC751A2734F3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{C5D5DF43-D68A-448F-BEE9-BC751A2734F3}"/>
   </bookViews>
   <sheets>
     <sheet name="All Time Distributions" sheetId="2" r:id="rId1"/>
@@ -490,7 +490,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7B78790-86BB-4A67-A9C4-9289D98D0CB3}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
@@ -506,6 +506,226 @@
       </c>
       <c r="C1" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>4310</v>
+      </c>
+      <c r="B2">
+        <v>71.833333333333329</v>
+      </c>
+      <c r="C2">
+        <v>1.1972222222222222</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>4945</v>
+      </c>
+      <c r="B3">
+        <v>82.416666666666671</v>
+      </c>
+      <c r="C3">
+        <v>1.3736111111111111</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>9577</v>
+      </c>
+      <c r="B4">
+        <v>159.61666666666667</v>
+      </c>
+      <c r="C4">
+        <v>2.660277777777778</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2154</v>
+      </c>
+      <c r="B5">
+        <v>35.9</v>
+      </c>
+      <c r="C5">
+        <v>0.59833333333333338</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>8434</v>
+      </c>
+      <c r="B6">
+        <v>140.56666666666666</v>
+      </c>
+      <c r="C6">
+        <v>2.3427777777777776</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>2275</v>
+      </c>
+      <c r="B7">
+        <v>37.916666666666664</v>
+      </c>
+      <c r="C7">
+        <v>0.63194444444444442</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>3617</v>
+      </c>
+      <c r="B8">
+        <v>60.283333333333331</v>
+      </c>
+      <c r="C8">
+        <v>1.0047222222222223</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>3973</v>
+      </c>
+      <c r="B9">
+        <v>66.216666666666669</v>
+      </c>
+      <c r="C9">
+        <v>1.1036111111111111</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>4176</v>
+      </c>
+      <c r="B10">
+        <v>69.599999999999994</v>
+      </c>
+      <c r="C10">
+        <v>1.1599999999999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>2741</v>
+      </c>
+      <c r="B11">
+        <v>45.68333333333333</v>
+      </c>
+      <c r="C11">
+        <v>0.76138888888888889</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>4504</v>
+      </c>
+      <c r="B12">
+        <v>75.066666666666663</v>
+      </c>
+      <c r="C12">
+        <v>1.2511111111111111</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>3101</v>
+      </c>
+      <c r="B13">
+        <v>51.68333333333333</v>
+      </c>
+      <c r="C13">
+        <v>0.86138888888888887</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>2570</v>
+      </c>
+      <c r="B14">
+        <v>42.833333333333336</v>
+      </c>
+      <c r="C14">
+        <v>0.71388888888888891</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>8032</v>
+      </c>
+      <c r="B15">
+        <v>133.86666666666667</v>
+      </c>
+      <c r="C15">
+        <v>2.2311111111111113</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>3689</v>
+      </c>
+      <c r="B16">
+        <v>61.483333333333334</v>
+      </c>
+      <c r="C16">
+        <v>1.0247222222222223</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>2972</v>
+      </c>
+      <c r="B17">
+        <v>49.533333333333331</v>
+      </c>
+      <c r="C17">
+        <v>0.8255555555555556</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>5762</v>
+      </c>
+      <c r="B18">
+        <v>96.033333333333331</v>
+      </c>
+      <c r="C18">
+        <v>1.6005555555555555</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>2936</v>
+      </c>
+      <c r="B19">
+        <v>48.93333333333333</v>
+      </c>
+      <c r="C19">
+        <v>0.81555555555555559</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>7288</v>
+      </c>
+      <c r="B20">
+        <v>121.46666666666667</v>
+      </c>
+      <c r="C20">
+        <v>2.0244444444444443</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>6307</v>
+      </c>
+      <c r="B21">
+        <v>105.11666666666666</v>
+      </c>
+      <c r="C21">
+        <v>1.7519444444444445</v>
       </c>
     </row>
   </sheetData>

</xml_diff>